<commit_message>
updated to allow both create and update of procedures and steps. (#771)
* updated to allow both create and update of procedures and steps.

* Adding Export

Co-authored-by: jamesbridgeford <james.bridgeford@protonmail.ch>
</commit_message>
<xml_diff>
--- a/MSR.UI/MSR.UI.Answer/src/assets/CsvFiles/ProceduresSample.xlsx
+++ b/MSR.UI/MSR.UI.Answer/src/assets/CsvFiles/ProceduresSample.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd4f18a707bfc9ba/Desktop/Ticket Attachments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FreeLance\CMH\Answer3.0\MSR.UI\MSR.UI.Answer\src\assets\CsvFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{614EA611-4AA4-40C9-9D68-4DD70B6D64B9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48875410-42D7-4549-854E-F9B7A94AE728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="13620" windowHeight="10065" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PROC_STEP_EXPORT" sheetId="1" r:id="rId1"/>
-    <sheet name="PROCEDURE_NAME_EXPORT" sheetId="2" r:id="rId2"/>
+    <sheet name="Procedures" sheetId="2" r:id="rId1"/>
+    <sheet name="ProcedureSteps" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -29,54 +29,60 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
-  <si>
-    <t>PROCEDURE_ID</t>
-  </si>
-  <si>
-    <t>PROCEDURE_NAME</t>
-  </si>
-  <si>
-    <t>STEP_TEXT</t>
-  </si>
-  <si>
-    <t>PRINT_ORDER</t>
-  </si>
-  <si>
-    <t>REF_DOC_ID</t>
-  </si>
-  <si>
-    <t>COMMENT</t>
-  </si>
-  <si>
-    <t>STEP_TIME</t>
-  </si>
-  <si>
-    <t>EXTRA_NOTE1</t>
-  </si>
-  <si>
-    <t>SERIALIZE</t>
-  </si>
-  <si>
-    <t>DEFAULT_ROLE_ID</t>
-  </si>
-  <si>
-    <t>SUCCESS_MONITOR</t>
-  </si>
-  <si>
-    <t>INTERNAL_LOCATION</t>
-  </si>
-  <si>
-    <t>LOC_TYPE</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>Title</t>
   </si>
   <si>
-    <t>ANS_ID</t>
-  </si>
-  <si>
-    <t>PROC_TYPE_ID</t>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>Revision</t>
+  </si>
+  <si>
+    <t>ProcedureId</t>
+  </si>
+  <si>
+    <t>StepText</t>
+  </si>
+  <si>
+    <t>ProcedureStepTypeId</t>
+  </si>
+  <si>
+    <t>PrintOrder</t>
+  </si>
+  <si>
+    <t>LaborTime</t>
+  </si>
+  <si>
+    <t>EquipmentTime</t>
+  </si>
+  <si>
+    <t>ReplacementCost</t>
+  </si>
+  <si>
+    <t>Utilization</t>
+  </si>
+  <si>
+    <t>UsefulLife</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>ProcedureType</t>
+  </si>
+  <si>
+    <t>DurationType</t>
+  </si>
+  <si>
+    <t>ProcedureName</t>
   </si>
 </sst>
 </file>
@@ -565,13 +571,11 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="37" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="37" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="1" builtinId="30" customBuiltin="1"/>
@@ -927,63 +931,44 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="16.85546875" customWidth="1"/>
-    <col min="4" max="4" width="35.42578125" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" customWidth="1"/>
-    <col min="10" max="10" width="21.85546875" customWidth="1"/>
-    <col min="11" max="11" width="21.140625" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L1" t="s">
-        <v>12</v>
-      </c>
-      <c r="M1" t="s">
-        <v>13</v>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -993,32 +978,61 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D2" s="1"/>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>